<commit_message>
Dodaje plik interfejsu: -BookInterface
Dodaje zmienną do GlobalVariables:
-UserID

Dodałem register do LoginInterface
Poprawiłem kod w moich plikach
</commit_message>
<xml_diff>
--- a/DATABASE/bookNew.xlsx
+++ b/DATABASE/bookNew.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30105"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30110"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\working\waccache\FR1PEPF00001169\EXCELCNV\65d635ba-622d-4214-8c40-bd9c21ababd3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{73590EE6-0A71-4553-95B8-9448309E4A13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DA60D7CB-0065-43BF-A6BC-971827DF2C9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-60" yWindow="-60" windowWidth="15480" windowHeight="11640" xr2:uid="{6502C133-150D-4F54-88C8-31CE5A5F8E12}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>ID</t>
   </si>
@@ -72,6 +72,12 @@
   </si>
   <si>
     <t>The Object-Oriented Thought Process</t>
+  </si>
+  <si>
+    <t>Andrzej Sapkowski</t>
+  </si>
+  <si>
+    <t>Wiedźmin: Ostatnie życzenie</t>
   </si>
 </sst>
 </file>
@@ -931,7 +937,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60826CDF-661A-4289-9A79-FA33799C86AD}">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11.42578125" customWidth="1"/>
@@ -1022,6 +1028,26 @@
         <v>43177</v>
       </c>
     </row>
+    <row r="5" spans="1:6">
+      <c r="A5">
+        <v>104</v>
+      </c>
+      <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5">
+        <v>1500</v>
+      </c>
+      <c r="E5" s="1">
+        <v>43174</v>
+      </c>
+      <c r="F5" s="1">
+        <v>43174</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>